<commit_message>
W01 D3 companion and workbook: headings and tab titles ask their question, glossary cites the new slides
The companion's section and experiment headings are questions, the guided walk's steps and chapter
map carry the six chapter questions, and the glossary gains ERP, extract, tie out and booked value
with every slide and notebook reference moved to the rebuilt decks. The workbook's tabs are titled
by the question each settles, its start tab says who Anand and his analyst are, and INV-01 and the
profile's first amount move from Rs 2,400 to Rs 2,500, as chapter 2 and experiment A already did, so
no invented value echoes the take-home's refund; the recalc manifest's total follows to Rs 20,300.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015wSjC19kt2ddCVrsoGpR6H
</commit_message>
<xml_diff>
--- a/content/W01/D3/demos/C2_W01_D03_decision_tool_STUDENT.xlsx
+++ b/content/W01/D3/demos/C2_W01_D03_decision_tool_STUDENT.xlsx
@@ -490,14 +490,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Which Q1 figure is right: the decision tool</t>
+          <t>Which four cleaning decisions get the export to the books?</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Kalpa Retail, Week 1, Wednesday. Four cleaning decisions the day taught, one tab each, and an Export tab that assembles the note to Anand.</t>
+          <t>Kalpa Retail, Week 1, Wednesday. Anand Iyer, the finance controller, acts only on a figure that matches his books to the rupee, and his analyst ties out every figure, matching it to the books line by line. Four cleaning decisions the day taught get an export there, one tab each, and an Export tab assembles the note.</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>2400</t>
+          <t>2500</t>
         </is>
       </c>
       <c r="B5">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2400</v>
+        <v>2500</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2400</v>
+        <v>2500</v>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
@@ -1114,7 +1114,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Keep the large order?</t>
+          <t>Should the large order stay in revenue?</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Rows and rupees, to the books</t>
+          <t>Do rows and rupees both tie to the books?</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The note, assembled</t>
+          <t>Is the note to Anand ready to paste?</t>
         </is>
       </c>
     </row>

</xml_diff>